<commit_message>
fix: parse raw data with correct decimal handling, restoring true truck volumes
The raw MDPI supplement stores each record as a single semicolon-separated
string inside the .xls sheet. The old pipeline split it with read_csv2(),
whose European locale treats the period as a grouping mark. This stripped
decimal points from the data: truck volumes of 2.5, 6.5, and 7.2 cubic
meters became 25, 65, and 72, and coordinates had to be repaired with an
ad-hoc string hack that re-inserted the period into longitudes.

Reading the semicolon-separated values with read_delim(delim = ";") and a
standard decimal mark fixes 12 of 35 truck volumes to their true source
values and makes the coordinate workarounds unnecessary. trips is verified
identical to the previous build; only trucks volumes change. The commented
out codebook block is removed and the script follows tidyverse style.
</commit_message>
<xml_diff>
--- a/inst/extdata/trucks.xlsx
+++ b/inst/extdata/trucks.xlsx
@@ -472,7 +472,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>35</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>36</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="6">
@@ -528,7 +528,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="n">
-        <v>65</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="11">
@@ -536,7 +536,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="n">
-        <v>36</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="12">
@@ -560,7 +560,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="n">
-        <v>65</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="15">
@@ -600,7 +600,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="n">
-        <v>37</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="20">
@@ -632,7 +632,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="n">
-        <v>27</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="24">
@@ -648,7 +648,7 @@
         <v>25</v>
       </c>
       <c r="B25" t="n">
-        <v>36</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="26">
@@ -664,7 +664,7 @@
         <v>27</v>
       </c>
       <c r="B27" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="28">
@@ -680,7 +680,7 @@
         <v>29</v>
       </c>
       <c r="B29" t="n">
-        <v>37</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="30">
@@ -696,7 +696,7 @@
         <v>31</v>
       </c>
       <c r="B31" t="n">
-        <v>72</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="32">
@@ -728,7 +728,7 @@
         <v>35</v>
       </c>
       <c r="B35" t="n">
-        <v>72</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="36">

</xml_diff>

<commit_message>
fix: recode transposed AUS numberplates to UAS and store fid as integer
Ugandan numberplates start with U; the raw data records AUS 088V, AUS 892G,
and AUS 119X alongside UAS counterparts carrying identical truck volumes,
so the AUS prefix is a transposition. Recoding merges trucks from 35 to 33
unique plates and updates 458 trips rows. fid is integer-valued and now
stored as integer; dictionary.csv updated and reordered accordingly.
</commit_message>
<xml_diff>
--- a/inst/extdata/trucks.xlsx
+++ b/inst/extdata/trucks.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">numberplate</t>
   </si>
@@ -20,7 +20,7 @@
     <t xml:space="preserve">volume</t>
   </si>
   <si>
-    <t xml:space="preserve">AUS 119X</t>
+    <t xml:space="preserve">UAS 119X</t>
   </si>
   <si>
     <t xml:space="preserve">UAG 448X</t>
@@ -44,7 +44,7 @@
     <t xml:space="preserve">UAT 767H</t>
   </si>
   <si>
-    <t xml:space="preserve">AUS 088V</t>
+    <t xml:space="preserve">UAS 088V</t>
   </si>
   <si>
     <t xml:space="preserve">UAJ 874D</t>
@@ -56,9 +56,6 @@
     <t xml:space="preserve">UAV 754B</t>
   </si>
   <si>
-    <t xml:space="preserve">UAS 088V</t>
-  </si>
-  <si>
     <t xml:space="preserve">LG 0366-01</t>
   </si>
   <si>
@@ -107,7 +104,7 @@
     <t xml:space="preserve">UAJ 866Z</t>
   </si>
   <si>
-    <t xml:space="preserve">AUS 892G</t>
+    <t xml:space="preserve">UAS 892G</t>
   </si>
   <si>
     <t xml:space="preserve">UAT 845E</t>
@@ -117,9 +114,6 @@
   </si>
   <si>
     <t xml:space="preserve">UAH 706D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UAS 892G</t>
   </si>
   <si>
     <t xml:space="preserve">LG 0257-01</t>
@@ -560,7 +554,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -576,7 +570,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -592,7 +586,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="19">
@@ -600,7 +594,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -608,7 +602,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -624,7 +618,7 @@
         <v>22</v>
       </c>
       <c r="B22" t="n">
-        <v>10</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="23">
@@ -632,7 +626,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -640,7 +634,7 @@
         <v>24</v>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="25">
@@ -648,7 +642,7 @@
         <v>25</v>
       </c>
       <c r="B25" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
@@ -656,7 +650,7 @@
         <v>26</v>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="27">
@@ -664,7 +658,7 @@
         <v>27</v>
       </c>
       <c r="B27" t="n">
-        <v>2.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
@@ -672,7 +666,7 @@
         <v>28</v>
       </c>
       <c r="B28" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="29">
@@ -680,7 +674,7 @@
         <v>29</v>
       </c>
       <c r="B29" t="n">
-        <v>3.7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30">
@@ -688,7 +682,7 @@
         <v>30</v>
       </c>
       <c r="B30" t="n">
-        <v>10</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="31">
@@ -696,7 +690,7 @@
         <v>31</v>
       </c>
       <c r="B31" t="n">
-        <v>7.2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32">
@@ -704,7 +698,7 @@
         <v>32</v>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -712,7 +706,7 @@
         <v>33</v>
       </c>
       <c r="B33" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
@@ -720,22 +714,6 @@
         <v>34</v>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35" t="n">
-        <v>7.2</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s">
-        <v>36</v>
-      </c>
-      <c r="B36" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>